<commit_message>
add new measurement and modeling threaded rod
</commit_message>
<xml_diff>
--- a/Measurements/ADDA-Series45 M6, Series 45 molded in insert/batch02/ADDA-Series45.xlsx
+++ b/Measurements/ADDA-Series45 M6, Series 45 molded in insert/batch02/ADDA-Series45.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manoe\Meng\solidworks\Measurements\ADDA-Series45 M6, Series 45 molded in insert\batch02\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EE5B643-D42F-4882-8429-955248333758}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C96A1F3-8A83-4A9A-A4E5-61BB52734FEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{32BFC42B-CD3D-49FE-8254-52B3F518DB85}"/>
   </bookViews>
@@ -153,13 +153,13 @@
     <t>M6, Series 45 Molded in Insert</t>
   </si>
   <si>
-    <t>3/4/2026</t>
-  </si>
-  <si>
     <t>Radius</t>
   </si>
   <si>
     <t>Angle</t>
+  </si>
+  <si>
+    <t>3/10/2026</t>
   </si>
 </sst>
 </file>
@@ -2623,7 +2623,7 @@
         <v>1</v>
       </c>
       <c r="F1" s="26" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G1" s="35" t="s">
         <v>22</v>
@@ -2823,7 +2823,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C7" s="6">
         <v>0.01</v>
@@ -2888,11 +2888,21 @@
       <c r="H8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
+      <c r="I8" s="2">
+        <v>0.48799999999999999</v>
+      </c>
+      <c r="J8" s="2">
+        <v>0.48759999999999998</v>
+      </c>
+      <c r="K8" s="2">
+        <v>0.4864</v>
+      </c>
+      <c r="L8" s="2">
+        <v>0.48749999999999999</v>
+      </c>
+      <c r="M8" s="2">
+        <v>0.48649999999999999</v>
+      </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
@@ -2921,11 +2931,21 @@
       <c r="H9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
+      <c r="I9" s="2">
+        <v>0.35920000000000002</v>
+      </c>
+      <c r="J9" s="2">
+        <v>0.35949999999999999</v>
+      </c>
+      <c r="K9" s="2">
+        <v>0.35780000000000001</v>
+      </c>
+      <c r="L9" s="2">
+        <v>0.36030000000000001</v>
+      </c>
+      <c r="M9" s="2">
+        <v>0.35720000000000002</v>
+      </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
@@ -2954,11 +2974,21 @@
       <c r="H10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-      <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
+      <c r="I10" s="2">
+        <v>0.3165</v>
+      </c>
+      <c r="J10" s="2">
+        <v>0.31719999999999998</v>
+      </c>
+      <c r="K10" s="2">
+        <v>0.31509999999999999</v>
+      </c>
+      <c r="L10" s="2">
+        <v>0.31769999999999998</v>
+      </c>
+      <c r="M10" s="2">
+        <v>0.31290000000000001</v>
+      </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
@@ -2987,11 +3017,21 @@
       <c r="H11" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
-      <c r="M11" s="2"/>
+      <c r="I11" s="2">
+        <v>0.35410000000000003</v>
+      </c>
+      <c r="J11" s="2">
+        <v>0.3548</v>
+      </c>
+      <c r="K11" s="2">
+        <v>0.35449999999999998</v>
+      </c>
+      <c r="L11" s="2">
+        <v>0.35399999999999998</v>
+      </c>
+      <c r="M11" s="2">
+        <v>0.35489999999999999</v>
+      </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
@@ -3020,11 +3060,21 @@
       <c r="H12" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
-      <c r="K12" s="2"/>
-      <c r="L12" s="2"/>
-      <c r="M12" s="2"/>
+      <c r="I12" s="2">
+        <v>6.9699999999999998E-2</v>
+      </c>
+      <c r="J12" s="2">
+        <v>6.8099999999999994E-2</v>
+      </c>
+      <c r="K12" s="2">
+        <v>7.2300000000000003E-2</v>
+      </c>
+      <c r="L12" s="2">
+        <v>7.1199999999999999E-2</v>
+      </c>
+      <c r="M12" s="2">
+        <v>7.1900000000000006E-2</v>
+      </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="4">
@@ -3053,11 +3103,21 @@
       <c r="H13" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2"/>
-      <c r="M13" s="2"/>
+      <c r="I13" s="2">
+        <v>8.1000000000000003E-2</v>
+      </c>
+      <c r="J13" s="2">
+        <v>7.9000000000000001E-2</v>
+      </c>
+      <c r="K13" s="2">
+        <v>8.0799999999999997E-2</v>
+      </c>
+      <c r="L13" s="2">
+        <v>7.7600000000000002E-2</v>
+      </c>
+      <c r="M13" s="2">
+        <v>8.3799999999999999E-2</v>
+      </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="4">
@@ -3086,11 +3146,21 @@
       <c r="H14" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
-      <c r="L14" s="2"/>
-      <c r="M14" s="2"/>
+      <c r="I14" s="2">
+        <v>0.123</v>
+      </c>
+      <c r="J14" s="2">
+        <v>0.122</v>
+      </c>
+      <c r="K14" s="2">
+        <v>0.1232</v>
+      </c>
+      <c r="L14" s="2">
+        <v>0.1265</v>
+      </c>
+      <c r="M14" s="2">
+        <v>0.11550000000000001</v>
+      </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
@@ -3119,11 +3189,21 @@
       <c r="H15" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
-      <c r="L15" s="2"/>
-      <c r="M15" s="2"/>
+      <c r="I15" s="2">
+        <v>0.14199999999999999</v>
+      </c>
+      <c r="J15" s="2">
+        <v>0.14410000000000001</v>
+      </c>
+      <c r="K15" s="2">
+        <v>0.1424</v>
+      </c>
+      <c r="L15" s="2">
+        <v>0.14449999999999999</v>
+      </c>
+      <c r="M15" s="2">
+        <v>0.14030000000000001</v>
+      </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="4">
@@ -3152,18 +3232,28 @@
       <c r="H16" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
-      <c r="L16" s="2"/>
-      <c r="M16" s="2"/>
+      <c r="I16" s="2">
+        <v>9.11E-2</v>
+      </c>
+      <c r="J16" s="2">
+        <v>9.0300000000000005E-2</v>
+      </c>
+      <c r="K16" s="2">
+        <v>9.0499999999999997E-2</v>
+      </c>
+      <c r="L16" s="2">
+        <v>8.9700000000000002E-2</v>
+      </c>
+      <c r="M16" s="2">
+        <v>9.1999999999999998E-2</v>
+      </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="4">
         <v>13</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C17" s="6">
         <v>24</v>
@@ -3185,13 +3275,23 @@
       <c r="H17" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
-      <c r="L17" s="2"/>
-      <c r="M17" s="2"/>
+      <c r="I17" s="2">
+        <v>23.991599999999998</v>
+      </c>
+      <c r="J17" s="2">
+        <v>24.035699999999999</v>
+      </c>
+      <c r="K17" s="2">
+        <v>23.978300000000001</v>
+      </c>
+      <c r="L17" s="2">
+        <v>24.072299999999998</v>
+      </c>
+      <c r="M17" s="2">
+        <v>24.060500000000001</v>
+      </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4">
         <v>14</v>
       </c>

</xml_diff>